<commit_message>
feat: tlumaczenia opisow (desc) modulow zawierajacych polskie slowa
- itemDesc() — opisy przechodza przez PRODUCT_TERMS jak nazwy/grupy;
  opisy czysto techniczne (5V / dif / ...) bez wpisu = identyczne
- 11 opisow z polskimi slowami (gora/dol, podlaczanie, PWM, RTD...)
  przetlumaczone roboczo na LT i LV
- ceny_EUR_LT_LV.xlsx: nowe kolumny Opis LT / Opis LV (do weryfikacji)
- tlumaczenia_LT_LV.xlsx: dopisane wiersze opisow (spojnosc zrodel)

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/ceny_EUR_LT_LV.xlsx
+++ b/ceny_EUR_LT_LV.xlsx
@@ -467,7 +467,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A12"/>
+  <dimension ref="A1:A13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="110" customWidth="1" min="1" max="1"/>
@@ -521,29 +521,36 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>4. Nazwy LT/LV to robocze tłumaczenia — popraw bezpośrednio w komórce, jeśli są błędne.</t>
+          <t>4. Nazwy LT/LV oraz Opisy LT/LV to robocze tłumaczenia — popraw bezpośrednio w komórce, jeśli błędne.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Kolumna 'Nr katalogowy' (zamrożona po lewej) to odniesienie, czego dotyczy dana nazwa.</t>
+          <t xml:space="preserve">   Opisy czysto techniczne (np. '5V / dif / 32b / 250kHz') są identyczne we wszystkich językach.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
+          <t xml:space="preserve">   Kolumna 'Nr katalogowy' (zamrożona po lewej) to odniesienie, czego dotyczy dana nazwa/opis.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
           <t>5. Arkusz 'Zestaw bazowy' — cena kompletnego zestawu startowego w EUR (w PL: 1 000,00 zł).</t>
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" t="inlineStr"/>
-    </row>
     <row r="12">
-      <c r="A12" t="inlineStr">
+      <c r="A12" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
         <is>
           <t>Nie zmieniaj kolumny 'Nr katalogowy' ani nazw arkuszy — służą do automatycznego wczytania danych.</t>
         </is>
@@ -560,7 +567,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I23"/>
+  <dimension ref="A1:K23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -570,8 +577,10 @@
     <col width="14" customWidth="1" min="5" max="5"/>
     <col width="32" customWidth="1" min="6" max="6"/>
     <col width="32" customWidth="1" min="7" max="7"/>
-    <col width="16" customWidth="1" min="8" max="8"/>
-    <col width="16" customWidth="1" min="9" max="9"/>
+    <col width="32" customWidth="1" min="8" max="8"/>
+    <col width="32" customWidth="1" min="9" max="9"/>
+    <col width="16" customWidth="1" min="10" max="10"/>
+    <col width="16" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -592,7 +601,7 @@
       </c>
       <c r="D1" s="2" t="inlineStr">
         <is>
-          <t>Opis techniczny</t>
+          <t>Opis PL</t>
         </is>
       </c>
       <c r="E1" s="2" t="inlineStr">
@@ -612,10 +621,20 @@
       </c>
       <c r="H1" s="3" t="inlineStr">
         <is>
+          <t>Opis LT (do weryfikacji)</t>
+        </is>
+      </c>
+      <c r="I1" s="3" t="inlineStr">
+        <is>
+          <t>Opis LV (do weryfikacji)</t>
+        </is>
+      </c>
+      <c r="J1" s="3" t="inlineStr">
+        <is>
           <t>Cena promo EUR — LT (WYPEŁNIJ)</t>
         </is>
       </c>
-      <c r="I1" s="3" t="inlineStr">
+      <c r="K1" s="3" t="inlineStr">
         <is>
           <t>Cena promo EUR — LV (WYPEŁNIJ)</t>
         </is>
@@ -655,8 +674,18 @@
           <t>Inkrementālā enkodera modulis</t>
         </is>
       </c>
-      <c r="H2" s="7" t="n"/>
-      <c r="I2" s="7" t="n"/>
+      <c r="H2" s="6" t="inlineStr">
+        <is>
+          <t>5V / 422 / diff / 16b / 1000kHz</t>
+        </is>
+      </c>
+      <c r="I2" s="6" t="inlineStr">
+        <is>
+          <t>5V / 422 / diff / 16b / 1000kHz</t>
+        </is>
+      </c>
+      <c r="J2" s="7" t="n"/>
+      <c r="K2" s="7" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="4" t="inlineStr">
@@ -692,8 +721,18 @@
           <t>Inkrementālā enkodera modulis</t>
         </is>
       </c>
-      <c r="H3" s="7" t="n"/>
-      <c r="I3" s="7" t="n"/>
+      <c r="H3" s="6" t="inlineStr">
+        <is>
+          <t>5..24V / uni / 16b / 1000kHz</t>
+        </is>
+      </c>
+      <c r="I3" s="6" t="inlineStr">
+        <is>
+          <t>5..24V / uni / 16b / 1000kHz</t>
+        </is>
+      </c>
+      <c r="J3" s="7" t="n"/>
+      <c r="K3" s="7" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="4" t="inlineStr">
@@ -729,8 +768,18 @@
           <t>Inkrementālā enkodera modulis</t>
         </is>
       </c>
-      <c r="H4" s="7" t="n"/>
-      <c r="I4" s="7" t="n"/>
+      <c r="H4" s="6" t="inlineStr">
+        <is>
+          <t>5..24V / uni / 16b / 1000kHz</t>
+        </is>
+      </c>
+      <c r="I4" s="6" t="inlineStr">
+        <is>
+          <t>5..24V / uni / 16b / 1000kHz</t>
+        </is>
+      </c>
+      <c r="J4" s="7" t="n"/>
+      <c r="K4" s="7" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
@@ -766,8 +815,18 @@
           <t>Inkrementālā enkodera modulis</t>
         </is>
       </c>
-      <c r="H5" s="7" t="n"/>
-      <c r="I5" s="7" t="n"/>
+      <c r="H5" s="6" t="inlineStr">
+        <is>
+          <t>5V / dif / 32b / 250kHz</t>
+        </is>
+      </c>
+      <c r="I5" s="6" t="inlineStr">
+        <is>
+          <t>5V / dif / 32b / 250kHz</t>
+        </is>
+      </c>
+      <c r="J5" s="7" t="n"/>
+      <c r="K5" s="7" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
@@ -803,8 +862,18 @@
           <t>Inkrementālā enkodera modulis</t>
         </is>
       </c>
-      <c r="H6" s="7" t="n"/>
-      <c r="I6" s="7" t="n"/>
+      <c r="H6" s="6" t="inlineStr">
+        <is>
+          <t>24V / dif / 32b / 250kHz</t>
+        </is>
+      </c>
+      <c r="I6" s="6" t="inlineStr">
+        <is>
+          <t>24V / dif / 32b / 250kHz</t>
+        </is>
+      </c>
+      <c r="J6" s="7" t="n"/>
+      <c r="K6" s="7" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
@@ -840,8 +909,18 @@
           <t>Inkrementālā enkodera modulis</t>
         </is>
       </c>
-      <c r="H7" s="7" t="n"/>
-      <c r="I7" s="7" t="n"/>
+      <c r="H7" s="6" t="inlineStr">
+        <is>
+          <t>24V / se / 32b / 250kHz</t>
+        </is>
+      </c>
+      <c r="I7" s="6" t="inlineStr">
+        <is>
+          <t>24V / se / 32b / 250kHz</t>
+        </is>
+      </c>
+      <c r="J7" s="7" t="n"/>
+      <c r="K7" s="7" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
@@ -877,8 +956,18 @@
           <t>Inkrementālā enkodera modulis</t>
         </is>
       </c>
-      <c r="H8" s="7" t="n"/>
-      <c r="I8" s="7" t="n"/>
+      <c r="H8" s="6" t="inlineStr">
+        <is>
+          <t>5V / dif / 32b / 250kHz</t>
+        </is>
+      </c>
+      <c r="I8" s="6" t="inlineStr">
+        <is>
+          <t>5V / dif / 32b / 250kHz</t>
+        </is>
+      </c>
+      <c r="J8" s="7" t="n"/>
+      <c r="K8" s="7" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
@@ -914,8 +1003,18 @@
           <t>Inkrementālā enkodera modulis</t>
         </is>
       </c>
-      <c r="H9" s="7" t="n"/>
-      <c r="I9" s="7" t="n"/>
+      <c r="H9" s="6" t="inlineStr">
+        <is>
+          <t>24V / se / 32b / 250kHz</t>
+        </is>
+      </c>
+      <c r="I9" s="6" t="inlineStr">
+        <is>
+          <t>24V / se / 32b / 250kHz</t>
+        </is>
+      </c>
+      <c r="J9" s="7" t="n"/>
+      <c r="K9" s="7" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
@@ -951,8 +1050,18 @@
           <t>Skaitītājs uz augšu/leju</t>
         </is>
       </c>
-      <c r="H10" s="7" t="n"/>
-      <c r="I10" s="7" t="n"/>
+      <c r="H10" s="6" t="inlineStr">
+        <is>
+          <t>24V, aukštyn/žemyn, 100kHz</t>
+        </is>
+      </c>
+      <c r="I10" s="6" t="inlineStr">
+        <is>
+          <t>24V, uz augšu/leju, 100kHz</t>
+        </is>
+      </c>
+      <c r="J10" s="7" t="n"/>
+      <c r="K10" s="7" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
@@ -988,8 +1097,18 @@
           <t>Skaitītājs uz augšu</t>
         </is>
       </c>
-      <c r="H11" s="7" t="n"/>
-      <c r="I11" s="7" t="n"/>
+      <c r="H11" s="6" t="inlineStr">
+        <is>
+          <t>24V, aukštyn, su blokavimu</t>
+        </is>
+      </c>
+      <c r="I11" s="6" t="inlineStr">
+        <is>
+          <t>24V, uz augšu, ar bloķēšanu</t>
+        </is>
+      </c>
+      <c r="J11" s="7" t="n"/>
+      <c r="K11" s="7" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="4" t="inlineStr">
@@ -1025,8 +1144,18 @@
           <t>Frekvences skaitītājs</t>
         </is>
       </c>
-      <c r="H12" s="7" t="n"/>
-      <c r="I12" s="7" t="n"/>
+      <c r="H12" s="6" t="inlineStr">
+        <is>
+          <t>0,1–100kHz</t>
+        </is>
+      </c>
+      <c r="I12" s="6" t="inlineStr">
+        <is>
+          <t>0,1–100kHz</t>
+        </is>
+      </c>
+      <c r="J12" s="7" t="n"/>
+      <c r="K12" s="7" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="4" t="inlineStr">
@@ -1062,8 +1191,18 @@
           <t>Skaitītājs uz augšu/leju</t>
         </is>
       </c>
-      <c r="H13" s="7" t="n"/>
-      <c r="I13" s="7" t="n"/>
+      <c r="H13" s="6" t="inlineStr">
+        <is>
+          <t>aukštyn/žemyn, su skaitmeniniu išėjimu</t>
+        </is>
+      </c>
+      <c r="I13" s="6" t="inlineStr">
+        <is>
+          <t>uz augšu/leju, ar digitālo izeju</t>
+        </is>
+      </c>
+      <c r="J13" s="7" t="n"/>
+      <c r="K13" s="7" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="4" t="inlineStr">
@@ -1099,8 +1238,18 @@
           <t>Skaitītājs uz augšu</t>
         </is>
       </c>
-      <c r="H14" s="7" t="n"/>
-      <c r="I14" s="7" t="n"/>
+      <c r="H14" s="6" t="inlineStr">
+        <is>
+          <t>2x aukštyn, 16bit</t>
+        </is>
+      </c>
+      <c r="I14" s="6" t="inlineStr">
+        <is>
+          <t>2x uz augšu, 16bit</t>
+        </is>
+      </c>
+      <c r="J14" s="7" t="n"/>
+      <c r="K14" s="7" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="4" t="inlineStr">
@@ -1136,8 +1285,18 @@
           <t>Skaitītājs uz augšu/leju</t>
         </is>
       </c>
-      <c r="H15" s="7" t="n"/>
-      <c r="I15" s="7" t="n"/>
+      <c r="H15" s="6" t="inlineStr">
+        <is>
+          <t>24V, 2x aukštyn/žemyn, 16bit, 500Hz</t>
+        </is>
+      </c>
+      <c r="I15" s="6" t="inlineStr">
+        <is>
+          <t>24V, 2x uz augšu/leju, 16bit, 500Hz</t>
+        </is>
+      </c>
+      <c r="J15" s="7" t="n"/>
+      <c r="K15" s="7" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="4" t="inlineStr">
@@ -1173,8 +1332,18 @@
           <t>Soļu motoru vadības modulis</t>
         </is>
       </c>
-      <c r="H16" s="7" t="n"/>
-      <c r="I16" s="7" t="n"/>
+      <c r="H16" s="6" t="inlineStr">
+        <is>
+          <t>RS-422/24 V DC; 20 mA</t>
+        </is>
+      </c>
+      <c r="I16" s="6" t="inlineStr">
+        <is>
+          <t>RS-422/24 V DC; 20 mA</t>
+        </is>
+      </c>
+      <c r="J16" s="7" t="n"/>
+      <c r="K16" s="7" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="4" t="inlineStr">
@@ -1210,8 +1379,18 @@
           <t>Soļu motoru vadības modulis</t>
         </is>
       </c>
-      <c r="H17" s="7" t="n"/>
-      <c r="I17" s="7" t="n"/>
+      <c r="H17" s="6" t="inlineStr">
+        <is>
+          <t>24 V DC; 1,5 A</t>
+        </is>
+      </c>
+      <c r="I17" s="6" t="inlineStr">
+        <is>
+          <t>24 V DC; 1,5 A</t>
+        </is>
+      </c>
+      <c r="J17" s="7" t="n"/>
+      <c r="K17" s="7" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="4" t="inlineStr">
@@ -1247,8 +1426,18 @@
           <t>Soļu motoru vadības modulis</t>
         </is>
       </c>
-      <c r="H18" s="7" t="n"/>
-      <c r="I18" s="7" t="n"/>
+      <c r="H18" s="6" t="inlineStr">
+        <is>
+          <t>70 V DC; 7,5 A</t>
+        </is>
+      </c>
+      <c r="I18" s="6" t="inlineStr">
+        <is>
+          <t>70 V DC; 7,5 A</t>
+        </is>
+      </c>
+      <c r="J18" s="7" t="n"/>
+      <c r="K18" s="7" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="4" t="inlineStr">
@@ -1284,8 +1473,18 @@
           <t>PWM modulis</t>
         </is>
       </c>
-      <c r="H19" s="7" t="n"/>
-      <c r="I19" s="7" t="n"/>
+      <c r="H19" s="6" t="inlineStr">
+        <is>
+          <t>2 išėjimai su impulso pločio reguliavimu (PWM)</t>
+        </is>
+      </c>
+      <c r="I19" s="6" t="inlineStr">
+        <is>
+          <t>2 izejas ar impulsa platuma regulēšanu (PWM)</t>
+        </is>
+      </c>
+      <c r="J19" s="7" t="n"/>
+      <c r="K19" s="7" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="4" t="inlineStr">
@@ -1321,8 +1520,18 @@
           <t>Proporcionālo vārstu modulis</t>
         </is>
       </c>
-      <c r="H20" s="7" t="n"/>
-      <c r="I20" s="7" t="n"/>
+      <c r="H20" s="6" t="inlineStr">
+        <is>
+          <t>2, 3, 4 laidų prijungimas</t>
+        </is>
+      </c>
+      <c r="I20" s="6" t="inlineStr">
+        <is>
+          <t>2, 3, 4 vadu pieslēgums</t>
+        </is>
+      </c>
+      <c r="J20" s="7" t="n"/>
+      <c r="K20" s="7" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="4" t="inlineStr">
@@ -1358,8 +1567,18 @@
           <t>Safety modulis</t>
         </is>
       </c>
-      <c r="H21" s="7" t="n"/>
-      <c r="I21" s="7" t="n"/>
+      <c r="H21" s="6" t="inlineStr">
+        <is>
+          <t>4FDI/2FDO; PROFIsafe; logika</t>
+        </is>
+      </c>
+      <c r="I21" s="6" t="inlineStr">
+        <is>
+          <t>4FDI/2FDO; PROFIsafe; loģika</t>
+        </is>
+      </c>
+      <c r="J21" s="7" t="n"/>
+      <c r="K21" s="7" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="4" t="inlineStr">
@@ -1395,8 +1614,18 @@
           <t>Safety modulis</t>
         </is>
       </c>
-      <c r="H22" s="7" t="n"/>
-      <c r="I22" s="7" t="n"/>
+      <c r="H22" s="6" t="inlineStr">
+        <is>
+          <t>4FDI/4FDO; PROFIsafe; logika</t>
+        </is>
+      </c>
+      <c r="I22" s="6" t="inlineStr">
+        <is>
+          <t>4FDI/4FDO; PROFIsafe; loģika</t>
+        </is>
+      </c>
+      <c r="J22" s="7" t="n"/>
+      <c r="K22" s="7" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="4" t="inlineStr">
@@ -1432,8 +1661,18 @@
           <t>RS-232/-485 saskarnes modulis</t>
         </is>
       </c>
-      <c r="H23" s="7" t="n"/>
-      <c r="I23" s="7" t="n"/>
+      <c r="H23" s="6" t="inlineStr">
+        <is>
+          <t>RS-232/RS-485</t>
+        </is>
+      </c>
+      <c r="I23" s="6" t="inlineStr">
+        <is>
+          <t>RS-232/RS-485</t>
+        </is>
+      </c>
+      <c r="J23" s="7" t="n"/>
+      <c r="K23" s="7" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1446,7 +1685,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H7"/>
+  <dimension ref="A1:J7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -1455,8 +1694,10 @@
     <col width="14" customWidth="1" min="4" max="4"/>
     <col width="32" customWidth="1" min="5" max="5"/>
     <col width="32" customWidth="1" min="6" max="6"/>
-    <col width="16" customWidth="1" min="7" max="7"/>
-    <col width="16" customWidth="1" min="8" max="8"/>
+    <col width="32" customWidth="1" min="7" max="7"/>
+    <col width="32" customWidth="1" min="8" max="8"/>
+    <col width="16" customWidth="1" min="9" max="9"/>
+    <col width="16" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1472,7 +1713,7 @@
       </c>
       <c r="C1" s="2" t="inlineStr">
         <is>
-          <t>Opis techniczny</t>
+          <t>Opis PL</t>
         </is>
       </c>
       <c r="D1" s="2" t="inlineStr">
@@ -1492,10 +1733,20 @@
       </c>
       <c r="G1" s="3" t="inlineStr">
         <is>
+          <t>Opis LT (do weryfikacji)</t>
+        </is>
+      </c>
+      <c r="H1" s="3" t="inlineStr">
+        <is>
+          <t>Opis LV (do weryfikacji)</t>
+        </is>
+      </c>
+      <c r="I1" s="3" t="inlineStr">
+        <is>
           <t>Cena promo EUR — LT (WYPEŁNIJ)</t>
         </is>
       </c>
-      <c r="H1" s="3" t="inlineStr">
+      <c r="J1" s="3" t="inlineStr">
         <is>
           <t>Cena promo EUR — LV (WYPEŁNIJ)</t>
         </is>
@@ -1530,8 +1781,18 @@
           <t>Digitālo ieeju modulis</t>
         </is>
       </c>
-      <c r="G2" s="7" t="n"/>
-      <c r="H2" s="7" t="n"/>
+      <c r="G2" s="6" t="inlineStr">
+        <is>
+          <t>16 DI 24V DC</t>
+        </is>
+      </c>
+      <c r="H2" s="6" t="inlineStr">
+        <is>
+          <t>16 DI 24V DC</t>
+        </is>
+      </c>
+      <c r="I2" s="7" t="n"/>
+      <c r="J2" s="7" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="4" t="inlineStr">
@@ -1562,8 +1823,18 @@
           <t>Digitālo izeju modulis</t>
         </is>
       </c>
-      <c r="G3" s="7" t="n"/>
-      <c r="H3" s="7" t="n"/>
+      <c r="G3" s="6" t="inlineStr">
+        <is>
+          <t>16 DO 24V DC 0,5A</t>
+        </is>
+      </c>
+      <c r="H3" s="6" t="inlineStr">
+        <is>
+          <t>16 DO 24V DC 0,5A</t>
+        </is>
+      </c>
+      <c r="I3" s="7" t="n"/>
+      <c r="J3" s="7" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="4" t="inlineStr">
@@ -1594,8 +1865,18 @@
           <t>Analogo ieeju modulis</t>
         </is>
       </c>
-      <c r="G4" s="7" t="n"/>
-      <c r="H4" s="7" t="n"/>
+      <c r="G4" s="6" t="inlineStr">
+        <is>
+          <t>4 AI RTD, 2, 3, 4 laidų</t>
+        </is>
+      </c>
+      <c r="H4" s="6" t="inlineStr">
+        <is>
+          <t>4 AI RTD, 2, 3, 4 vadu</t>
+        </is>
+      </c>
+      <c r="I4" s="7" t="n"/>
+      <c r="J4" s="7" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
@@ -1626,8 +1907,18 @@
           <t>Analogo ieeju modulis</t>
         </is>
       </c>
-      <c r="G5" s="7" t="n"/>
-      <c r="H5" s="7" t="n"/>
+      <c r="G5" s="6" t="inlineStr">
+        <is>
+          <t>8 AI 0/4–20mA</t>
+        </is>
+      </c>
+      <c r="H5" s="6" t="inlineStr">
+        <is>
+          <t>8 AI 0/4–20mA</t>
+        </is>
+      </c>
+      <c r="I5" s="7" t="n"/>
+      <c r="J5" s="7" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
@@ -1658,8 +1949,18 @@
           <t>Analogo ieeju modulis</t>
         </is>
       </c>
-      <c r="G6" s="7" t="n"/>
-      <c r="H6" s="7" t="n"/>
+      <c r="G6" s="6" t="inlineStr">
+        <is>
+          <t>8 AI 0–10V / ±10V DC</t>
+        </is>
+      </c>
+      <c r="H6" s="6" t="inlineStr">
+        <is>
+          <t>8 AI 0–10V / ±10V DC</t>
+        </is>
+      </c>
+      <c r="I6" s="7" t="n"/>
+      <c r="J6" s="7" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
@@ -1690,8 +1991,18 @@
           <t>Analogo izeju modulis</t>
         </is>
       </c>
-      <c r="G7" s="7" t="n"/>
-      <c r="H7" s="7" t="n"/>
+      <c r="G7" s="6" t="inlineStr">
+        <is>
+          <t>4 AO konfigūruojami įtampos/srovės (U/I)</t>
+        </is>
+      </c>
+      <c r="H7" s="6" t="inlineStr">
+        <is>
+          <t>4 AO konfigurējamas sprieguma/strāvas (U/I)</t>
+        </is>
+      </c>
+      <c r="I7" s="7" t="n"/>
+      <c r="J7" s="7" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>